<commit_message>
copia de seguridad de codigo y su conectada
</commit_message>
<xml_diff>
--- a/datos_samm/Equipos(2).xlsx
+++ b/datos_samm/Equipos(2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Analista Contable\Desktop\Dino-erp\datos_samm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80B3202F-5C56-4E23-B6CC-52870EE78864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA72260-B299-45AE-BC1E-4669EEC5EA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3500,9 +3500,12 @@
   <dimension ref="A1:U217"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="26.85546875" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" customWidth="1"/>
     <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.28515625" customWidth="1"/>
+    <col min="11" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>